<commit_message>
Weight table: clean title, add Train time column + params caption
</commit_message>
<xml_diff>
--- a/Weight_loss_Simulation/weight_study_v2_table.xlsx
+++ b/Weight_loss_Simulation/weight_study_v2_table.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,10 @@
     </font>
     <font>
       <i val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00B00000"/>
     </font>
   </fonts>
   <fills count="5">
@@ -82,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -97,6 +101,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -474,7 +479,8 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,6 +531,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Train time (s)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>In noise band?</t>
         </is>
       </c>
@@ -560,6 +571,7 @@
         <v>0.06469999999999999</v>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -591,7 +603,8 @@
       <c r="I3" s="3" t="n">
         <v>0.0557</v>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -627,7 +640,8 @@
       <c r="I4" s="3" t="n">
         <v>0.0586</v>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -663,7 +677,8 @@
       <c r="I5" s="4" t="n">
         <v>0.0535</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -700,6 +715,7 @@
         <v>0.06370000000000001</v>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -732,6 +748,7 @@
         <v>0.0674</v>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -763,7 +780,8 @@
       <c r="I8" s="3" t="n">
         <v>0.058</v>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -773,6 +791,20 @@
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Selected: C2 (0.5, 1.5, 1.0) - best measured RMSE and inside the noise band on hidden; C4 has the single lowest hidden but is statistically tied with C2, C3, C7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>All cases use the same 4x100 architecture (32,912 parameters), 2000 epochs on the same dataset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Train-time column is blank until wstudy_v2_log.txt is pulled from the cluster into this folder, then re-run this script.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weight table: fill Train time column from cluster log
</commit_message>
<xml_diff>
--- a/Weight_loss_Simulation/weight_study_v2_table.xlsx
+++ b/Weight_loss_Simulation/weight_study_v2_table.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +31,6 @@
     </font>
     <font>
       <i val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00B00000"/>
     </font>
   </fonts>
   <fills count="5">
@@ -86,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -101,7 +97,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -570,7 +565,9 @@
       <c r="I2" s="2" t="n">
         <v>0.06469999999999999</v>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>2118</v>
+      </c>
       <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -603,7 +600,9 @@
       <c r="I3" s="3" t="n">
         <v>0.0557</v>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="n">
+        <v>2096</v>
+      </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -640,7 +639,9 @@
       <c r="I4" s="3" t="n">
         <v>0.0586</v>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="n">
+        <v>2105</v>
+      </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -677,7 +678,9 @@
       <c r="I5" s="4" t="n">
         <v>0.0535</v>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="n">
+        <v>2104</v>
+      </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -714,7 +717,9 @@
       <c r="I6" s="2" t="n">
         <v>0.06370000000000001</v>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
+        <v>2107</v>
+      </c>
       <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
@@ -747,7 +752,9 @@
       <c r="I7" s="2" t="n">
         <v>0.0674</v>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>2095</v>
+      </c>
       <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
@@ -780,7 +787,9 @@
       <c r="I8" s="3" t="n">
         <v>0.058</v>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="n">
+        <v>2091</v>
+      </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
           <t>yes</t>
@@ -798,13 +807,6 @@
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>All cases use the same 4x100 architecture (32,912 parameters), 2000 epochs on the same dataset.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Train-time column is blank until wstudy_v2_log.txt is pulled from the cluster into this folder, then re-run this script.</t>
         </is>
       </c>
     </row>

</xml_diff>